<commit_message>
chore: archive one-off scripts, fix indentation, ignore .serena
</commit_message>
<xml_diff>
--- a/data/test_cases.xlsx
+++ b/data/test_cases.xlsx
@@ -553,14 +553,14 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="F4" t="n">
         <v>-1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>用户未找到</t>
+          <t>用户名或密码错误</t>
         </is>
       </c>
     </row>
@@ -586,14 +586,14 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="F5" t="n">
         <v>-1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>用户未找到</t>
+          <t>用户名或密码错误</t>
         </is>
       </c>
     </row>

</xml_diff>